<commit_message>
test(CT003): complete problem user defect execution
</commit_message>
<xml_diff>
--- a/docs/QA_Test_Plan.xlsx
+++ b/docs/QA_Test_Plan.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="362">
   <si>
     <t>This document was exported from Numbers.  Each table was converted to an Excel worksheet. All other objects on each Numbers sheet were placed on separate worksheets. Please be aware that formula calculations may differ in Excel.</t>
   </si>
@@ -651,6 +651,9 @@
     <t>problem_user / pethub123</t>
   </si>
   <si>
+    <t>The selected sorting option changed, but the order of the inventory items remained unchanged. This behavior was reproduced as expected for the `problem_user` defect persona.</t>
+  </si>
+  <si>
     <t>Add a Birds item to the cart.</t>
   </si>
   <si>
@@ -658,6 +661,9 @@
   </si>
   <si>
     <t>problem_user / pethub123; Birds item</t>
+  </si>
+  <si>
+    <t>The success message was displayed after attempting to add a Birds category pet, but the pet was not added to the cart.</t>
   </si>
   <si>
     <t>Open the cart.</t>
@@ -669,16 +675,25 @@
     <t>problem_user / pethub123; missing last name</t>
   </si>
   <si>
+    <t>The cart was opened successfully, but the previously selected Birds category pet was not present in the cart.</t>
+  </si>
+  <si>
     <t>Begin checkout and leave Last Name blank.</t>
   </si>
   <si>
     <t>The system rejects the order and displays the documented validation message.</t>
   </si>
   <si>
+    <t>Checkout submission was blocked when the Last Name field was left blank, and the expected validation message was displayed.</t>
+  </si>
+  <si>
     <t>Submit valid checkout data with a last name included.</t>
   </si>
   <si>
     <t>Checkout still fails because the last name is dropped in the documented problem_user flow.</t>
+  </si>
+  <si>
+    <t>After entering a last name, checkout submission still failed because the server dropped the Last Name value for the `problem_user` persona.</t>
   </si>
   <si>
     <t>Log in as performance_user.</t>
@@ -4339,7 +4354,7 @@
     </row>
     <row r="15">
       <c r="B15" t="s" s="3">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
@@ -4350,12 +4365,12 @@
         <v>5</v>
       </c>
       <c r="D16" t="s" s="5">
-        <v>262</v>
+        <v>267</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" t="s" s="3">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
@@ -4366,12 +4381,12 @@
         <v>5</v>
       </c>
       <c r="D18" t="s" s="5">
-        <v>290</v>
+        <v>295</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" t="s" s="3">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
@@ -4382,12 +4397,12 @@
         <v>5</v>
       </c>
       <c r="D20" t="s" s="5">
-        <v>313</v>
+        <v>318</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" t="s" s="3">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
@@ -4398,12 +4413,12 @@
         <v>5</v>
       </c>
       <c r="D22" t="s" s="5">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="23">
       <c r="B23" t="s" s="3">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
@@ -4414,7 +4429,7 @@
         <v>5</v>
       </c>
       <c r="D24" t="s" s="5">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
   </sheetData>
@@ -26545,9 +26560,11 @@
         <v>205</v>
       </c>
       <c r="F17" s="56"/>
-      <c r="G17" s="56"/>
+      <c r="G17" t="s" s="54">
+        <v>206</v>
+      </c>
       <c r="H17" t="s" s="54">
-        <v>58</v>
+        <v>159</v>
       </c>
       <c r="I17" s="54"/>
     </row>
@@ -26559,18 +26576,20 @@
         <v>2</v>
       </c>
       <c r="C18" t="s" s="57">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D18" t="s" s="57">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E18" t="s" s="57">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F18" s="59"/>
-      <c r="G18" s="59"/>
+      <c r="G18" t="s" s="57">
+        <v>210</v>
+      </c>
       <c r="H18" t="s" s="57">
-        <v>58</v>
+        <v>159</v>
       </c>
       <c r="I18" s="57"/>
     </row>
@@ -26582,18 +26601,20 @@
         <v>3</v>
       </c>
       <c r="C19" t="s" s="54">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D19" t="s" s="54">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E19" t="s" s="54">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="F19" s="56"/>
-      <c r="G19" s="56"/>
+      <c r="G19" t="s" s="54">
+        <v>214</v>
+      </c>
       <c r="H19" t="s" s="54">
-        <v>58</v>
+        <v>159</v>
       </c>
       <c r="I19" s="54"/>
     </row>
@@ -26605,18 +26626,20 @@
         <v>4</v>
       </c>
       <c r="C20" t="s" s="54">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="D20" t="s" s="54">
+        <v>216</v>
+      </c>
+      <c r="E20" t="s" s="54">
         <v>213</v>
       </c>
-      <c r="E20" t="s" s="54">
-        <v>211</v>
-      </c>
       <c r="F20" s="56"/>
-      <c r="G20" s="56"/>
+      <c r="G20" t="s" s="54">
+        <v>217</v>
+      </c>
       <c r="H20" t="s" s="54">
-        <v>58</v>
+        <v>159</v>
       </c>
       <c r="I20" s="54"/>
     </row>
@@ -26628,18 +26651,20 @@
         <v>5</v>
       </c>
       <c r="C21" t="s" s="54">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="D21" t="s" s="54">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="E21" t="s" s="54">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="F21" s="56"/>
-      <c r="G21" s="56"/>
+      <c r="G21" t="s" s="54">
+        <v>220</v>
+      </c>
       <c r="H21" t="s" s="54">
-        <v>58</v>
+        <v>159</v>
       </c>
       <c r="I21" s="54"/>
     </row>
@@ -26651,13 +26676,13 @@
         <v>1</v>
       </c>
       <c r="C22" t="s" s="57">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="D22" t="s" s="57">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="E22" t="s" s="57">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="F22" s="59"/>
       <c r="G22" s="59"/>
@@ -26674,13 +26699,13 @@
         <v>2</v>
       </c>
       <c r="C23" t="s" s="54">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="D23" t="s" s="54">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="E23" t="s" s="54">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="F23" s="56"/>
       <c r="G23" s="56"/>
@@ -26697,13 +26722,13 @@
         <v>1</v>
       </c>
       <c r="C24" t="s" s="57">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="D24" t="s" s="57">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="E24" t="s" s="57">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="F24" s="59"/>
       <c r="G24" s="59"/>
@@ -26720,13 +26745,13 @@
         <v>2</v>
       </c>
       <c r="C25" t="s" s="54">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="D25" t="s" s="54">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="E25" t="s" s="54">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="F25" s="56"/>
       <c r="G25" s="56"/>
@@ -26743,13 +26768,13 @@
         <v>1</v>
       </c>
       <c r="C26" t="s" s="57">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="D26" t="s" s="57">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="E26" t="s" s="57">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="F26" s="59"/>
       <c r="G26" s="59"/>
@@ -26766,13 +26791,13 @@
         <v>2</v>
       </c>
       <c r="C27" t="s" s="54">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="D27" t="s" s="54">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="E27" t="s" s="54">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="F27" s="56"/>
       <c r="G27" s="56"/>
@@ -26789,13 +26814,13 @@
         <v>3</v>
       </c>
       <c r="C28" t="s" s="57">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="D28" t="s" s="57">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="E28" t="s" s="57">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="F28" s="59"/>
       <c r="G28" s="59"/>
@@ -26812,13 +26837,13 @@
         <v>1</v>
       </c>
       <c r="C29" t="s" s="54">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="D29" t="s" s="54">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="E29" t="s" s="54">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="F29" s="56"/>
       <c r="G29" s="56"/>
@@ -26835,13 +26860,13 @@
         <v>2</v>
       </c>
       <c r="C30" t="s" s="57">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="D30" t="s" s="57">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="E30" t="s" s="57">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="F30" s="59"/>
       <c r="G30" s="59"/>
@@ -26858,13 +26883,13 @@
         <v>1</v>
       </c>
       <c r="C31" t="s" s="54">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="D31" t="s" s="54">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="E31" t="s" s="54">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="F31" s="56"/>
       <c r="G31" s="56"/>
@@ -26881,13 +26906,13 @@
         <v>2</v>
       </c>
       <c r="C32" t="s" s="57">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="D32" t="s" s="57">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="E32" t="s" s="57">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="F32" s="59"/>
       <c r="G32" s="59"/>
@@ -26904,13 +26929,13 @@
         <v>1</v>
       </c>
       <c r="C33" t="s" s="54">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="D33" t="s" s="54">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="E33" t="s" s="54">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="F33" s="56"/>
       <c r="G33" s="56"/>
@@ -26927,13 +26952,13 @@
         <v>2</v>
       </c>
       <c r="C34" t="s" s="57">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="D34" t="s" s="57">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="E34" t="s" s="57">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="F34" s="59"/>
       <c r="G34" s="59"/>
@@ -26950,13 +26975,13 @@
         <v>3</v>
       </c>
       <c r="C35" t="s" s="54">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="D35" t="s" s="54">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="E35" t="s" s="54">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="F35" s="56"/>
       <c r="G35" s="56"/>
@@ -26973,10 +26998,10 @@
         <v>1</v>
       </c>
       <c r="C36" t="s" s="57">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="D36" t="s" s="57">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="E36" t="s" s="57">
         <v>144</v>
@@ -26996,10 +27021,10 @@
         <v>2</v>
       </c>
       <c r="C37" t="s" s="54">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="D37" t="s" s="54">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="E37" t="s" s="54">
         <v>144</v>
@@ -27072,7 +27097,7 @@
   <sheetData>
     <row r="1" ht="15.55" customHeight="1">
       <c r="A1" t="s" s="36">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="B1" s="37"/>
       <c r="C1" s="38"/>
@@ -27089,13 +27114,13 @@
         <v>46</v>
       </c>
       <c r="B2" t="s" s="41">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="C2" t="s" s="41">
         <v>36</v>
       </c>
       <c r="D2" t="s" s="41">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="E2" t="s" s="41">
         <v>33</v>
@@ -27104,7 +27129,7 @@
         <v>40</v>
       </c>
       <c r="G2" t="s" s="41">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="H2" t="s" s="41">
         <v>48</v>
@@ -27119,13 +27144,13 @@
         <v>64</v>
       </c>
       <c r="B3" t="s" s="43">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="C3" t="s" s="43">
         <v>53</v>
       </c>
       <c r="D3" t="s" s="43">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="E3" t="s" s="43">
         <v>50</v>
@@ -27145,13 +27170,13 @@
         <v>64</v>
       </c>
       <c r="B4" t="s" s="45">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="C4" t="s" s="45">
         <v>68</v>
       </c>
       <c r="D4" t="s" s="45">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="E4" t="s" s="45">
         <v>66</v>
@@ -27171,13 +27196,13 @@
         <v>64</v>
       </c>
       <c r="B5" t="s" s="47">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="C5" t="s" s="47">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="D5" t="s" s="47">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="E5" t="s" s="47">
         <v>74</v>
@@ -27197,13 +27222,13 @@
         <v>64</v>
       </c>
       <c r="B6" t="s" s="45">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="C6" t="s" s="45">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="D6" t="s" s="45">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="E6" t="s" s="45">
         <v>83</v>
@@ -27223,13 +27248,13 @@
         <v>64</v>
       </c>
       <c r="B7" t="s" s="47">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="C7" t="s" s="47">
         <v>95</v>
       </c>
       <c r="D7" t="s" s="47">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="E7" t="s" s="47">
         <v>92</v>
@@ -27249,13 +27274,13 @@
         <v>64</v>
       </c>
       <c r="B8" t="s" s="45">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="C8" t="s" s="45">
         <v>105</v>
       </c>
       <c r="D8" t="s" s="45">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="E8" t="s" s="45">
         <v>102</v>
@@ -27275,13 +27300,13 @@
         <v>64</v>
       </c>
       <c r="B9" t="s" s="47">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="C9" t="s" s="47">
         <v>112</v>
       </c>
       <c r="D9" t="s" s="47">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="E9" t="s" s="47">
         <v>110</v>
@@ -27301,13 +27326,13 @@
         <v>64</v>
       </c>
       <c r="B10" t="s" s="45">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C10" t="s" s="45">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="D10" t="s" s="45">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="E10" t="s" s="45">
         <v>73</v>
@@ -27327,13 +27352,13 @@
         <v>64</v>
       </c>
       <c r="B11" t="s" s="47">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="C11" t="s" s="47">
         <v>131</v>
       </c>
       <c r="D11" t="s" s="47">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="E11" t="s" s="47">
         <v>128</v>
@@ -27353,13 +27378,13 @@
         <v>64</v>
       </c>
       <c r="B12" t="s" s="45">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="C12" t="s" s="45">
         <v>140</v>
       </c>
       <c r="D12" t="s" s="45">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="E12" t="s" s="45">
         <v>65</v>
@@ -27415,7 +27440,7 @@
   <sheetData>
     <row r="1" ht="15.55" customHeight="1">
       <c r="A1" t="s" s="36">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="B1" s="37"/>
       <c r="C1" s="38"/>
@@ -27430,19 +27455,19 @@
     </row>
     <row r="2" ht="20.05" customHeight="1">
       <c r="A2" t="s" s="41">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="B2" t="s" s="41">
         <v>33</v>
       </c>
       <c r="C2" t="s" s="41">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="D2" t="s" s="41">
         <v>15</v>
       </c>
       <c r="E2" t="s" s="41">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="F2" t="s" s="41">
         <v>41</v>
@@ -27465,7 +27490,7 @@
     </row>
     <row r="3" ht="25.55" customHeight="1">
       <c r="A3" t="s" s="43">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="B3" t="s" s="43">
         <v>50</v>
@@ -27474,31 +27499,31 @@
         <v>46281.958333333343</v>
       </c>
       <c r="D3" t="s" s="43">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="E3" t="s" s="43">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="F3" t="s" s="43">
         <v>159</v>
       </c>
       <c r="G3" t="s" s="43">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="H3" t="s" s="43">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="I3" s="44"/>
       <c r="J3" t="s" s="43">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="K3" t="s" s="43">
-        <v>300</v>
+        <v>305</v>
       </c>
     </row>
     <row r="4" ht="11.55" customHeight="1">
       <c r="A4" t="s" s="45">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="B4" t="s" s="45">
         <v>66</v>
@@ -27507,10 +27532,10 @@
         <v>46282.458333333336</v>
       </c>
       <c r="D4" t="s" s="45">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="E4" t="s" s="45">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="F4" t="s" s="45">
         <v>159</v>
@@ -27519,23 +27544,23 @@
       <c r="H4" s="46"/>
       <c r="I4" s="46"/>
       <c r="J4" t="s" s="45">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="K4" s="46"/>
     </row>
     <row r="5" ht="11.55" customHeight="1">
       <c r="A5" t="s" s="47">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="B5" t="s" s="47">
         <v>74</v>
       </c>
       <c r="C5" s="48"/>
       <c r="D5" t="s" s="47">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="E5" t="s" s="47">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="F5" t="s" s="47">
         <v>58</v>
@@ -27548,17 +27573,17 @@
     </row>
     <row r="6" ht="11.55" customHeight="1">
       <c r="A6" t="s" s="45">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="B6" t="s" s="45">
         <v>83</v>
       </c>
       <c r="C6" s="46"/>
       <c r="D6" t="s" s="45">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="E6" t="s" s="45">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="F6" t="s" s="45">
         <v>58</v>
@@ -27571,17 +27596,17 @@
     </row>
     <row r="7" ht="11.55" customHeight="1">
       <c r="A7" t="s" s="47">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="B7" t="s" s="47">
         <v>92</v>
       </c>
       <c r="C7" s="48"/>
       <c r="D7" t="s" s="47">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="E7" t="s" s="47">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="F7" t="s" s="47">
         <v>58</v>
@@ -27594,17 +27619,17 @@
     </row>
     <row r="8" ht="11.55" customHeight="1">
       <c r="A8" t="s" s="45">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="B8" t="s" s="45">
         <v>102</v>
       </c>
       <c r="C8" s="46"/>
       <c r="D8" t="s" s="45">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="E8" t="s" s="45">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="F8" t="s" s="45">
         <v>58</v>
@@ -27617,17 +27642,17 @@
     </row>
     <row r="9" ht="11.55" customHeight="1">
       <c r="A9" t="s" s="47">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="B9" t="s" s="47">
         <v>110</v>
       </c>
       <c r="C9" s="48"/>
       <c r="D9" t="s" s="47">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="E9" t="s" s="47">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="F9" t="s" s="47">
         <v>58</v>
@@ -27640,17 +27665,17 @@
     </row>
     <row r="10" ht="11.55" customHeight="1">
       <c r="A10" t="s" s="45">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="B10" t="s" s="45">
         <v>73</v>
       </c>
       <c r="C10" s="46"/>
       <c r="D10" t="s" s="45">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="E10" t="s" s="45">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="F10" t="s" s="45">
         <v>58</v>
@@ -27663,17 +27688,17 @@
     </row>
     <row r="11" ht="11.55" customHeight="1">
       <c r="A11" t="s" s="47">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="B11" t="s" s="47">
         <v>128</v>
       </c>
       <c r="C11" s="48"/>
       <c r="D11" t="s" s="47">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="E11" t="s" s="47">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="F11" t="s" s="47">
         <v>58</v>
@@ -27686,17 +27711,17 @@
     </row>
     <row r="12" ht="11.55" customHeight="1">
       <c r="A12" t="s" s="45">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="B12" t="s" s="45">
         <v>65</v>
       </c>
       <c r="C12" s="46"/>
       <c r="D12" t="s" s="45">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="E12" t="s" s="45">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="F12" t="s" s="45">
         <v>58</v>
@@ -40590,7 +40615,7 @@
   <sheetData>
     <row r="1" ht="15.55" customHeight="1">
       <c r="A1" t="s" s="36">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="B1" s="37"/>
       <c r="C1" s="38"/>
@@ -40620,10 +40645,10 @@
         <v>33</v>
       </c>
       <c r="D2" t="s" s="41">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="E2" t="s" s="41">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="F2" t="s" s="41">
         <v>38</v>
@@ -40638,7 +40663,7 @@
         <v>15</v>
       </c>
       <c r="J2" t="s" s="41">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="K2" t="s" s="41">
         <v>151</v>
@@ -40650,10 +40675,10 @@
         <v>152</v>
       </c>
       <c r="N2" t="s" s="41">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="O2" t="s" s="41">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="P2" t="s" s="41">
         <v>155</v>
@@ -59663,7 +59688,7 @@
   <sheetData>
     <row r="1" ht="15.55" customHeight="1">
       <c r="A1" t="s" s="36">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="B1" s="37"/>
       <c r="C1" s="38"/>
@@ -59678,13 +59703,13 @@
         <v>33</v>
       </c>
       <c r="B2" t="s" s="41">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="C2" t="s" s="41">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="D2" t="s" s="41">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="E2" t="s" s="41">
         <v>42</v>
@@ -59705,19 +59730,19 @@
         <v>57</v>
       </c>
       <c r="C3" t="s" s="43">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="D3" t="s" s="43">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="E3" t="s" s="43">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="F3" t="s" s="43">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="G3" t="s" s="43">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="H3" s="44"/>
     </row>
@@ -59729,19 +59754,19 @@
         <v>57</v>
       </c>
       <c r="C4" t="s" s="45">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="D4" t="s" s="45">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="E4" t="s" s="45">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="F4" t="s" s="45">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="G4" t="s" s="45">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="H4" s="46"/>
     </row>
@@ -59753,19 +59778,19 @@
         <v>57</v>
       </c>
       <c r="C5" t="s" s="47">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="D5" t="s" s="47">
+        <v>335</v>
+      </c>
+      <c r="E5" t="s" s="47">
         <v>330</v>
       </c>
-      <c r="E5" t="s" s="47">
-        <v>325</v>
-      </c>
       <c r="F5" t="s" s="47">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="G5" t="s" s="47">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="H5" s="48"/>
     </row>
@@ -59777,19 +59802,19 @@
         <v>57</v>
       </c>
       <c r="C6" t="s" s="45">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="D6" t="s" s="45">
+        <v>335</v>
+      </c>
+      <c r="E6" t="s" s="45">
         <v>330</v>
       </c>
-      <c r="E6" t="s" s="45">
-        <v>325</v>
-      </c>
       <c r="F6" t="s" s="45">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="G6" t="s" s="45">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="H6" s="46"/>
     </row>
@@ -59801,19 +59826,19 @@
         <v>57</v>
       </c>
       <c r="C7" t="s" s="47">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="D7" t="s" s="47">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="E7" t="s" s="47">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="F7" t="s" s="47">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="G7" t="s" s="47">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="H7" s="48"/>
     </row>
@@ -59825,19 +59850,19 @@
         <v>57</v>
       </c>
       <c r="C8" t="s" s="45">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="D8" t="s" s="45">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="E8" t="s" s="45">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="F8" t="s" s="45">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="G8" t="s" s="45">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="H8" s="46"/>
     </row>
@@ -59849,19 +59874,19 @@
         <v>57</v>
       </c>
       <c r="C9" t="s" s="47">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="D9" t="s" s="47">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="E9" t="s" s="47">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="F9" t="s" s="47">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="G9" t="s" s="47">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="H9" s="48"/>
     </row>
@@ -59873,19 +59898,19 @@
         <v>57</v>
       </c>
       <c r="C10" t="s" s="45">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="D10" t="s" s="45">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="E10" t="s" s="45">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="F10" t="s" s="45">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="G10" t="s" s="45">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="H10" s="46"/>
     </row>
@@ -59897,19 +59922,19 @@
         <v>133</v>
       </c>
       <c r="C11" t="s" s="47">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="D11" t="s" s="47">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="E11" t="s" s="47">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="F11" t="s" s="47">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="G11" t="s" s="47">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="H11" s="48"/>
     </row>
@@ -59921,19 +59946,19 @@
         <v>57</v>
       </c>
       <c r="C12" t="s" s="45">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="D12" t="s" s="45">
+        <v>335</v>
+      </c>
+      <c r="E12" t="s" s="45">
         <v>330</v>
       </c>
-      <c r="E12" t="s" s="45">
-        <v>325</v>
-      </c>
       <c r="F12" t="s" s="45">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="G12" t="s" s="45">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="H12" s="46"/>
     </row>
@@ -69859,7 +69884,7 @@
   <sheetData>
     <row r="1" ht="19.45" customHeight="1">
       <c r="A1" t="s" s="67">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B1" s="68"/>
       <c r="C1" s="68"/>
@@ -69897,7 +69922,7 @@
     </row>
     <row r="3" ht="19.55" customHeight="1">
       <c r="A3" t="s" s="71">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="B3" s="72">
         <f>COUNTA('Test Cases'!A3:A1000)</f>
@@ -69920,7 +69945,7 @@
     </row>
     <row r="4" ht="19.55" customHeight="1">
       <c r="A4" t="s" s="71">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="B4" s="72">
         <f>COUNTIF('Test Execution'!F3:F1000,"Pass")</f>
@@ -69943,7 +69968,7 @@
     </row>
     <row r="5" ht="19.55" customHeight="1">
       <c r="A5" t="s" s="71">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="B5" s="72">
         <f>COUNTIF('Test Execution'!F3:F1000,"Fail")</f>
@@ -69966,7 +69991,7 @@
     </row>
     <row r="6" ht="19.55" customHeight="1">
       <c r="A6" t="s" s="71">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="B6" s="72">
         <f>COUNTIF('Test Execution'!F3:F1000,"Blocked")</f>
@@ -69989,7 +70014,7 @@
     </row>
     <row r="7" ht="19.55" customHeight="1">
       <c r="A7" t="s" s="71">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="B7" s="72">
         <f>COUNTIF('Test Execution'!F3:F1000,"Skipped")</f>
@@ -70035,7 +70060,7 @@
     </row>
     <row r="9" ht="19.55" customHeight="1">
       <c r="A9" t="s" s="71">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="B9" s="72">
         <f>COUNTIF('Automation Mapping'!E3:E1000,"Automated")</f>
@@ -70058,7 +70083,7 @@
     </row>
     <row r="10" ht="19.55" customHeight="1">
       <c r="A10" t="s" s="71">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="B10" s="72">
         <f>COUNTIF('Defects'!H3:H1000,"Open")</f>
@@ -70081,7 +70106,7 @@
     </row>
     <row r="11" ht="19.55" customHeight="1">
       <c r="A11" t="s" s="71">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="B11" s="72">
         <f>COUNTIF('Defects'!F3:F1000,"Critical")</f>
@@ -70104,7 +70129,7 @@
     </row>
     <row r="12" ht="19.55" customHeight="1">
       <c r="A12" t="s" s="71">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="B12" s="73">
         <f>IF(B3=0,0,B3/B3)</f>
@@ -70127,7 +70152,7 @@
     </row>
     <row r="13" ht="19.55" customHeight="1">
       <c r="A13" t="s" s="71">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="B13" s="73">
         <f>IF(COUNTA('Automation Mapping'!A3:A1000)=0,0,B8/COUNTA('Automation Mapping'!A3:A1000))</f>
@@ -70243,7 +70268,7 @@
       <c r="J18" s="20"/>
       <c r="K18" s="20"/>
       <c r="L18" t="s" s="74">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="M18" s="76">
         <f>COUNTIF('Defects'!F3:F1000,"Critical")</f>
@@ -70258,7 +70283,7 @@
       <c r="B19" s="20"/>
       <c r="C19" s="20"/>
       <c r="D19" t="s" s="74">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="E19" s="75">
         <f>COUNTIF('Test Execution'!F3:F1000,"Fail")</f>
@@ -70291,7 +70316,7 @@
       <c r="B20" s="20"/>
       <c r="C20" s="20"/>
       <c r="D20" t="s" s="74">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="E20" s="75">
         <f>COUNTIF('Test Execution'!F3:F1000,"Blocked")</f>
@@ -70324,7 +70349,7 @@
       <c r="B21" s="20"/>
       <c r="C21" s="20"/>
       <c r="D21" t="s" s="74">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="E21" s="75">
         <f>COUNTIF('Test Execution'!F3:F1000,"Skipped")</f>
@@ -70342,7 +70367,7 @@
       <c r="J21" s="20"/>
       <c r="K21" s="20"/>
       <c r="L21" t="s" s="74">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="M21" s="76">
         <f>COUNTIF('Defects'!F3:F1000,"Low")</f>

</xml_diff>

<commit_message>
test: update execution results and notes for CT006
</commit_message>
<xml_diff>
--- a/docs/QA_Test_Plan.xlsx
+++ b/docs/QA_Test_Plan.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="456">
   <si>
     <t>This document was exported from Numbers.  Each table was converted to an Excel worksheet. All other objects on each Numbers sheet were placed on separate worksheets. Please be aware that formula calculations may differ in Excel.</t>
   </si>
@@ -833,7 +833,10 @@
     <t>The first booking step is visible and interaction begins normally.</t>
   </si>
   <si>
-    <t>clinic seed data</t>
+    <t>/clinic</t>
+  </si>
+  <si>
+    <t>Clinic booking wizard opened successfully at /clinic.</t>
   </si>
   <si>
     <t>Select a valid service and veterinarian.</t>
@@ -842,7 +845,10 @@
     <t>The booking progresses to date selection without errors.</t>
   </si>
   <si>
-    <t>valid service and vet selection</t>
+    <t>Valid available service; valid available veterinarian</t>
+  </si>
+  <si>
+    <t>Valid service and veterinarian were selected successfully, and the flow proceeded to the date and slot step.</t>
   </si>
   <si>
     <t>Submit a valid booking summary.</t>
@@ -851,7 +857,58 @@
     <t>The appointment is created and a confirmation is displayed.</t>
   </si>
   <si>
-    <t>valid booking data</t>
+    <t>Valid available date; valid available time slot</t>
+  </si>
+  <si>
+    <t>A valid date and available time slot were selected successfully.</t>
+  </si>
+  <si>
+    <t>Enter valid owner and pet details.</t>
+  </si>
+  <si>
+    <t>The details step accepts the values without validation errors.</t>
+  </si>
+  <si>
+    <t>Owner: John Smith; Email: john.smith@example.com; Pet: Buddy</t>
+  </si>
+  <si>
+    <t>Valid owner and pet details were entered without validation errors.</t>
+  </si>
+  <si>
+    <t>Review the summary.</t>
+  </si>
+  <si>
+    <t>All previously selected values are displayed accurately in the review step.</t>
+  </si>
+  <si>
+    <t>Previously selected service, veterinarian, date, time slot, owner, and pet details</t>
+  </si>
+  <si>
+    <t>Booking summary displayed the previously selected details accurately.</t>
+  </si>
+  <si>
+    <t>Submit the booking.</t>
+  </si>
+  <si>
+    <t>A confirmation page or success summary is shown with a valid booking reference.</t>
+  </si>
+  <si>
+    <t>Previously entered valid booking data</t>
+  </si>
+  <si>
+    <t>Booking was submitted successfully and a valid booking confirmation was displayed.</t>
+  </si>
+  <si>
+    <t>Open the appointments view.</t>
+  </si>
+  <si>
+    <t>The appointment is visible and matches the submitted booking details.</t>
+  </si>
+  <si>
+    <t>Booking reference generated in Step 6</t>
+  </si>
+  <si>
+    <t>The created appointment was visible in the appointments view and matched the submitted booking details.</t>
   </si>
   <si>
     <t>Attempt to continue with missing required clinic data.</t>
@@ -1179,10 +1236,16 @@
     <t>EXE-006</t>
   </si>
   <si>
-    <t>TBD</t>
+    <t>All 7 steps passed. The clinic booking workflow completed successfully with valid service, veterinarian, date, time slot, owner, and pet data. The appointment was created and verified in the appointments view.</t>
+  </si>
+  <si>
+    <t>Clinic booking flow worked as expected.</t>
   </si>
   <si>
     <t>EXE-007</t>
+  </si>
+  <si>
+    <t>TBD</t>
   </si>
   <si>
     <t>EXE-008</t>
@@ -2590,7 +2653,7 @@
               <c:numCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>7.000000</c:v>
+                  <c:v>8.000000</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.000000</c:v>
@@ -2602,7 +2665,7 @@
                   <c:v>0.000000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>5.000000</c:v>
+                  <c:v>4.000000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4601,7 +4664,7 @@
     </row>
     <row r="15">
       <c r="B15" t="s" s="3">
-        <v>326</v>
+        <v>345</v>
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
@@ -4612,12 +4675,12 @@
         <v>5</v>
       </c>
       <c r="D16" t="s" s="5">
-        <v>326</v>
+        <v>345</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" t="s" s="3">
-        <v>354</v>
+        <v>373</v>
       </c>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
@@ -4625,15 +4688,15 @@
     <row r="18">
       <c r="B18" s="4"/>
       <c r="C18" t="s" s="4">
-        <v>355</v>
+        <v>374</v>
       </c>
       <c r="D18" t="s" s="5">
-        <v>356</v>
+        <v>375</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" t="s" s="3">
-        <v>391</v>
+        <v>412</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
@@ -4644,12 +4707,12 @@
         <v>5</v>
       </c>
       <c r="D20" t="s" s="5">
-        <v>391</v>
+        <v>412</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" t="s" s="3">
-        <v>397</v>
+        <v>418</v>
       </c>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
@@ -4660,12 +4723,12 @@
         <v>5</v>
       </c>
       <c r="D22" t="s" s="5">
-        <v>397</v>
+        <v>418</v>
       </c>
     </row>
     <row r="23">
       <c r="B23" t="s" s="3">
-        <v>421</v>
+        <v>442</v>
       </c>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
@@ -4676,7 +4739,7 @@
         <v>5</v>
       </c>
       <c r="D24" t="s" s="5">
-        <v>421</v>
+        <v>442</v>
       </c>
     </row>
   </sheetData>
@@ -26411,7 +26474,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A2:I53"/>
+  <dimension ref="A2:I57"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="13.4" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6.23438" style="49" customWidth="1"/>
@@ -27210,9 +27273,11 @@
         <v>264</v>
       </c>
       <c r="F32" s="58"/>
-      <c r="G32" s="58"/>
+      <c r="G32" t="s" s="57">
+        <v>265</v>
+      </c>
       <c r="H32" t="s" s="57">
-        <v>98</v>
+        <v>58</v>
       </c>
       <c r="I32" s="57"/>
     </row>
@@ -27224,18 +27289,20 @@
         <v>2</v>
       </c>
       <c r="C33" t="s" s="60">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D33" t="s" s="60">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E33" t="s" s="60">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F33" s="61"/>
-      <c r="G33" s="61"/>
+      <c r="G33" t="s" s="60">
+        <v>269</v>
+      </c>
       <c r="H33" t="s" s="60">
-        <v>98</v>
+        <v>58</v>
       </c>
       <c r="I33" s="60"/>
     </row>
@@ -27247,128 +27314,138 @@
         <v>3</v>
       </c>
       <c r="C34" t="s" s="57">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="D34" t="s" s="57">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E34" t="s" s="57">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="F34" s="58"/>
-      <c r="G34" s="58"/>
+      <c r="G34" t="s" s="57">
+        <v>273</v>
+      </c>
       <c r="H34" t="s" s="57">
-        <v>98</v>
+        <v>58</v>
       </c>
       <c r="I34" s="57"/>
     </row>
     <row r="35" ht="24.55" customHeight="1">
       <c r="A35" t="s" s="55">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="B35" s="59">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C35" t="s" s="60">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D35" t="s" s="60">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="E35" t="s" s="60">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="F35" s="61"/>
-      <c r="G35" s="61"/>
+      <c r="G35" t="s" s="60">
+        <v>277</v>
+      </c>
       <c r="H35" t="s" s="60">
-        <v>98</v>
+        <v>58</v>
       </c>
       <c r="I35" s="60"/>
     </row>
     <row r="36" ht="24.55" customHeight="1">
       <c r="A36" t="s" s="55">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="B36" s="56">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C36" t="s" s="57">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="D36" t="s" s="57">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="E36" t="s" s="57">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="F36" s="58"/>
-      <c r="G36" s="58"/>
+      <c r="G36" t="s" s="57">
+        <v>281</v>
+      </c>
       <c r="H36" t="s" s="57">
-        <v>98</v>
+        <v>58</v>
       </c>
       <c r="I36" s="57"/>
     </row>
-    <row r="37" ht="11.55" customHeight="1">
+    <row r="37" ht="24.55" customHeight="1">
       <c r="A37" t="s" s="55">
-        <v>73</v>
+        <v>103</v>
       </c>
       <c r="B37" s="59">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C37" t="s" s="60">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="D37" t="s" s="60">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="E37" t="s" s="60">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="F37" s="61"/>
-      <c r="G37" s="61"/>
+      <c r="G37" t="s" s="60">
+        <v>285</v>
+      </c>
       <c r="H37" t="s" s="60">
-        <v>98</v>
+        <v>58</v>
       </c>
       <c r="I37" s="60"/>
     </row>
     <row r="38" ht="24.55" customHeight="1">
       <c r="A38" t="s" s="55">
-        <v>73</v>
+        <v>103</v>
       </c>
       <c r="B38" s="56">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C38" t="s" s="57">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="D38" t="s" s="57">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="E38" t="s" s="57">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="F38" s="58"/>
-      <c r="G38" s="58"/>
+      <c r="G38" t="s" s="57">
+        <v>289</v>
+      </c>
       <c r="H38" t="s" s="57">
-        <v>98</v>
+        <v>58</v>
       </c>
       <c r="I38" s="57"/>
     </row>
     <row r="39" ht="24.55" customHeight="1">
       <c r="A39" t="s" s="55">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="B39" s="59">
         <v>1</v>
       </c>
       <c r="C39" t="s" s="60">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="D39" t="s" s="60">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="E39" t="s" s="60">
-        <v>285</v>
+        <v>292</v>
       </c>
       <c r="F39" s="61"/>
       <c r="G39" s="61"/>
@@ -27379,19 +27456,19 @@
     </row>
     <row r="40" ht="24.55" customHeight="1">
       <c r="A40" t="s" s="55">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="B40" s="56">
         <v>2</v>
       </c>
       <c r="C40" t="s" s="57">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="D40" t="s" s="57">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="E40" t="s" s="57">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="F40" s="58"/>
       <c r="G40" s="58"/>
@@ -27400,21 +27477,21 @@
       </c>
       <c r="I40" s="57"/>
     </row>
-    <row r="41" ht="24.55" customHeight="1">
+    <row r="41" ht="11.55" customHeight="1">
       <c r="A41" t="s" s="55">
-        <v>129</v>
+        <v>73</v>
       </c>
       <c r="B41" s="59">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C41" t="s" s="60">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="D41" t="s" s="60">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="E41" t="s" s="60">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="F41" s="61"/>
       <c r="G41" s="61"/>
@@ -27423,103 +27500,95 @@
       </c>
       <c r="I41" s="60"/>
     </row>
-    <row r="42" ht="11.55" customHeight="1">
+    <row r="42" ht="24.55" customHeight="1">
       <c r="A42" t="s" s="55">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="B42" s="56">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s" s="57">
+        <v>299</v>
+      </c>
+      <c r="D42" t="s" s="57">
+        <v>300</v>
+      </c>
+      <c r="E42" t="s" s="57">
+        <v>301</v>
+      </c>
+      <c r="F42" s="58"/>
+      <c r="G42" s="58"/>
+      <c r="H42" t="s" s="57">
+        <v>98</v>
+      </c>
+      <c r="I42" s="57"/>
+    </row>
+    <row r="43" ht="24.55" customHeight="1">
+      <c r="A43" t="s" s="55">
+        <v>129</v>
+      </c>
+      <c r="B43" s="59">
         <v>1</v>
       </c>
-      <c r="C42" t="s" s="57">
-        <v>292</v>
-      </c>
-      <c r="D42" t="s" s="57">
-        <v>293</v>
-      </c>
-      <c r="E42" t="s" s="57">
-        <v>145</v>
-      </c>
-      <c r="F42" s="58"/>
-      <c r="G42" t="s" s="57">
-        <v>294</v>
-      </c>
-      <c r="H42" t="s" s="57">
-        <v>58</v>
-      </c>
-      <c r="I42" s="57"/>
-    </row>
-    <row r="43" ht="11.55" customHeight="1">
-      <c r="A43" t="s" s="55">
-        <v>65</v>
-      </c>
-      <c r="B43" s="59">
+      <c r="C43" t="s" s="60">
+        <v>302</v>
+      </c>
+      <c r="D43" t="s" s="60">
+        <v>303</v>
+      </c>
+      <c r="E43" t="s" s="60">
+        <v>304</v>
+      </c>
+      <c r="F43" s="61"/>
+      <c r="G43" s="61"/>
+      <c r="H43" t="s" s="60">
+        <v>98</v>
+      </c>
+      <c r="I43" s="60"/>
+    </row>
+    <row r="44" ht="24.55" customHeight="1">
+      <c r="A44" t="s" s="55">
+        <v>129</v>
+      </c>
+      <c r="B44" s="56">
         <v>2</v>
       </c>
-      <c r="C43" t="s" s="60">
-        <v>295</v>
-      </c>
-      <c r="D43" t="s" s="60">
-        <v>296</v>
-      </c>
-      <c r="E43" t="s" s="60">
-        <v>145</v>
-      </c>
-      <c r="F43" s="61"/>
-      <c r="G43" t="s" s="60">
-        <v>297</v>
-      </c>
-      <c r="H43" t="s" s="60">
-        <v>58</v>
-      </c>
-      <c r="I43" s="60"/>
-    </row>
-    <row r="44" ht="11.55" customHeight="1">
-      <c r="A44" t="s" s="55">
-        <v>65</v>
-      </c>
-      <c r="B44" s="56">
+      <c r="C44" t="s" s="57">
+        <v>305</v>
+      </c>
+      <c r="D44" t="s" s="57">
+        <v>306</v>
+      </c>
+      <c r="E44" t="s" s="57">
+        <v>307</v>
+      </c>
+      <c r="F44" s="58"/>
+      <c r="G44" s="58"/>
+      <c r="H44" t="s" s="57">
+        <v>98</v>
+      </c>
+      <c r="I44" s="57"/>
+    </row>
+    <row r="45" ht="24.55" customHeight="1">
+      <c r="A45" t="s" s="55">
+        <v>129</v>
+      </c>
+      <c r="B45" s="59">
         <v>3</v>
       </c>
-      <c r="C44" t="s" s="57">
-        <v>298</v>
-      </c>
-      <c r="D44" t="s" s="57">
-        <v>299</v>
-      </c>
-      <c r="E44" t="s" s="57">
-        <v>145</v>
-      </c>
-      <c r="F44" s="58"/>
-      <c r="G44" t="s" s="57">
-        <v>300</v>
-      </c>
-      <c r="H44" t="s" s="57">
-        <v>58</v>
-      </c>
-      <c r="I44" s="57"/>
-    </row>
-    <row r="45" ht="11.55" customHeight="1">
-      <c r="A45" t="s" s="55">
-        <v>65</v>
-      </c>
-      <c r="B45" s="59">
-        <v>4</v>
-      </c>
       <c r="C45" t="s" s="60">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="D45" t="s" s="60">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="E45" t="s" s="60">
-        <v>145</v>
+        <v>310</v>
       </c>
       <c r="F45" s="61"/>
-      <c r="G45" t="s" s="60">
-        <v>303</v>
-      </c>
+      <c r="G45" s="61"/>
       <c r="H45" t="s" s="60">
-        <v>58</v>
+        <v>98</v>
       </c>
       <c r="I45" s="60"/>
     </row>
@@ -27528,41 +27597,45 @@
         <v>65</v>
       </c>
       <c r="B46" s="56">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C46" t="s" s="57">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="D46" t="s" s="57">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="E46" t="s" s="57">
         <v>145</v>
       </c>
       <c r="F46" s="58"/>
       <c r="G46" t="s" s="57">
-        <v>306</v>
-      </c>
-      <c r="H46" s="58"/>
+        <v>313</v>
+      </c>
+      <c r="H46" t="s" s="57">
+        <v>58</v>
+      </c>
       <c r="I46" s="57"/>
     </row>
     <row r="47" ht="11.55" customHeight="1">
       <c r="A47" t="s" s="55">
-        <v>147</v>
+        <v>65</v>
       </c>
       <c r="B47" s="59">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C47" t="s" s="60">
-        <v>248</v>
+        <v>314</v>
       </c>
       <c r="D47" t="s" s="60">
-        <v>307</v>
-      </c>
-      <c r="E47" s="61"/>
+        <v>315</v>
+      </c>
+      <c r="E47" t="s" s="60">
+        <v>145</v>
+      </c>
       <c r="F47" s="61"/>
       <c r="G47" t="s" s="60">
-        <v>251</v>
+        <v>316</v>
       </c>
       <c r="H47" t="s" s="60">
         <v>58</v>
@@ -27571,21 +27644,23 @@
     </row>
     <row r="48" ht="11.55" customHeight="1">
       <c r="A48" t="s" s="55">
-        <v>147</v>
+        <v>65</v>
       </c>
       <c r="B48" s="56">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C48" t="s" s="57">
-        <v>308</v>
+        <v>317</v>
       </c>
       <c r="D48" t="s" s="57">
-        <v>309</v>
-      </c>
-      <c r="E48" s="58"/>
+        <v>318</v>
+      </c>
+      <c r="E48" t="s" s="57">
+        <v>145</v>
+      </c>
       <c r="F48" s="58"/>
       <c r="G48" t="s" s="57">
-        <v>310</v>
+        <v>319</v>
       </c>
       <c r="H48" t="s" s="57">
         <v>58</v>
@@ -27594,23 +27669,23 @@
     </row>
     <row r="49" ht="11.55" customHeight="1">
       <c r="A49" t="s" s="55">
-        <v>147</v>
+        <v>65</v>
       </c>
       <c r="B49" s="59">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C49" t="s" s="60">
-        <v>311</v>
+        <v>320</v>
       </c>
       <c r="D49" t="s" s="60">
-        <v>312</v>
+        <v>321</v>
       </c>
       <c r="E49" t="s" s="60">
-        <v>313</v>
+        <v>145</v>
       </c>
       <c r="F49" s="61"/>
       <c r="G49" t="s" s="60">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="H49" t="s" s="60">
         <v>58</v>
@@ -27619,25 +27694,25 @@
     </row>
     <row r="50" ht="11.55" customHeight="1">
       <c r="A50" t="s" s="55">
-        <v>147</v>
+        <v>65</v>
       </c>
       <c r="B50" s="56">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C50" t="s" s="57">
-        <v>315</v>
+        <v>323</v>
       </c>
       <c r="D50" t="s" s="57">
-        <v>316</v>
-      </c>
-      <c r="E50" s="58"/>
+        <v>324</v>
+      </c>
+      <c r="E50" t="s" s="57">
+        <v>145</v>
+      </c>
       <c r="F50" s="58"/>
       <c r="G50" t="s" s="57">
-        <v>317</v>
-      </c>
-      <c r="H50" t="s" s="57">
-        <v>58</v>
-      </c>
+        <v>325</v>
+      </c>
+      <c r="H50" s="58"/>
       <c r="I50" s="57"/>
     </row>
     <row r="51" ht="11.55" customHeight="1">
@@ -27645,18 +27720,18 @@
         <v>147</v>
       </c>
       <c r="B51" s="59">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C51" t="s" s="60">
-        <v>259</v>
+        <v>248</v>
       </c>
       <c r="D51" t="s" s="60">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="E51" s="61"/>
       <c r="F51" s="61"/>
       <c r="G51" t="s" s="60">
-        <v>319</v>
+        <v>251</v>
       </c>
       <c r="H51" t="s" s="60">
         <v>58</v>
@@ -27668,18 +27743,18 @@
         <v>147</v>
       </c>
       <c r="B52" s="56">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C52" t="s" s="57">
-        <v>320</v>
+        <v>327</v>
       </c>
       <c r="D52" t="s" s="57">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="E52" s="58"/>
       <c r="F52" s="58"/>
       <c r="G52" t="s" s="57">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="H52" t="s" s="57">
         <v>58</v>
@@ -27691,30 +27766,124 @@
         <v>147</v>
       </c>
       <c r="B53" s="59">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C53" t="s" s="60">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="D53" t="s" s="60">
-        <v>324</v>
-      </c>
-      <c r="E53" s="61"/>
+        <v>331</v>
+      </c>
+      <c r="E53" t="s" s="60">
+        <v>332</v>
+      </c>
       <c r="F53" s="61"/>
       <c r="G53" t="s" s="60">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="H53" t="s" s="60">
         <v>58</v>
       </c>
       <c r="I53" s="60"/>
+    </row>
+    <row r="54" ht="11.55" customHeight="1">
+      <c r="A54" t="s" s="55">
+        <v>147</v>
+      </c>
+      <c r="B54" s="56">
+        <v>4</v>
+      </c>
+      <c r="C54" t="s" s="57">
+        <v>334</v>
+      </c>
+      <c r="D54" t="s" s="57">
+        <v>335</v>
+      </c>
+      <c r="E54" s="58"/>
+      <c r="F54" s="58"/>
+      <c r="G54" t="s" s="57">
+        <v>336</v>
+      </c>
+      <c r="H54" t="s" s="57">
+        <v>58</v>
+      </c>
+      <c r="I54" s="57"/>
+    </row>
+    <row r="55" ht="11.55" customHeight="1">
+      <c r="A55" t="s" s="55">
+        <v>147</v>
+      </c>
+      <c r="B55" s="59">
+        <v>5</v>
+      </c>
+      <c r="C55" t="s" s="60">
+        <v>259</v>
+      </c>
+      <c r="D55" t="s" s="60">
+        <v>337</v>
+      </c>
+      <c r="E55" s="61"/>
+      <c r="F55" s="61"/>
+      <c r="G55" t="s" s="60">
+        <v>338</v>
+      </c>
+      <c r="H55" t="s" s="60">
+        <v>58</v>
+      </c>
+      <c r="I55" s="60"/>
+    </row>
+    <row r="56" ht="11.55" customHeight="1">
+      <c r="A56" t="s" s="55">
+        <v>147</v>
+      </c>
+      <c r="B56" s="56">
+        <v>6</v>
+      </c>
+      <c r="C56" t="s" s="57">
+        <v>339</v>
+      </c>
+      <c r="D56" t="s" s="57">
+        <v>340</v>
+      </c>
+      <c r="E56" s="58"/>
+      <c r="F56" s="58"/>
+      <c r="G56" t="s" s="57">
+        <v>341</v>
+      </c>
+      <c r="H56" t="s" s="57">
+        <v>58</v>
+      </c>
+      <c r="I56" s="57"/>
+    </row>
+    <row r="57" ht="11.55" customHeight="1">
+      <c r="A57" t="s" s="55">
+        <v>147</v>
+      </c>
+      <c r="B57" s="59">
+        <v>7</v>
+      </c>
+      <c r="C57" t="s" s="60">
+        <v>342</v>
+      </c>
+      <c r="D57" t="s" s="60">
+        <v>343</v>
+      </c>
+      <c r="E57" s="61"/>
+      <c r="F57" s="61"/>
+      <c r="G57" t="s" s="60">
+        <v>344</v>
+      </c>
+      <c r="H57" t="s" s="60">
+        <v>58</v>
+      </c>
+      <c r="I57" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3 H10:H53">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3 H10:H57">
       <formula1>"Not Run,Pass,Fail,Blocked,Skipped"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H4:H9">
@@ -27748,7 +27917,7 @@
   <sheetData>
     <row r="1" ht="15.55" customHeight="1">
       <c r="A1" t="s" s="36">
-        <v>327</v>
+        <v>346</v>
       </c>
       <c r="B1" s="37"/>
       <c r="C1" s="38"/>
@@ -27765,13 +27934,13 @@
         <v>46</v>
       </c>
       <c r="B2" t="s" s="41">
-        <v>328</v>
+        <v>347</v>
       </c>
       <c r="C2" t="s" s="41">
         <v>36</v>
       </c>
       <c r="D2" t="s" s="41">
-        <v>329</v>
+        <v>348</v>
       </c>
       <c r="E2" t="s" s="41">
         <v>33</v>
@@ -27780,7 +27949,7 @@
         <v>40</v>
       </c>
       <c r="G2" t="s" s="41">
-        <v>330</v>
+        <v>349</v>
       </c>
       <c r="H2" t="s" s="41">
         <v>48</v>
@@ -27795,13 +27964,13 @@
         <v>64</v>
       </c>
       <c r="B3" t="s" s="43">
-        <v>331</v>
+        <v>350</v>
       </c>
       <c r="C3" t="s" s="43">
         <v>53</v>
       </c>
       <c r="D3" t="s" s="43">
-        <v>332</v>
+        <v>351</v>
       </c>
       <c r="E3" t="s" s="43">
         <v>50</v>
@@ -27821,13 +27990,13 @@
         <v>64</v>
       </c>
       <c r="B4" t="s" s="45">
-        <v>333</v>
+        <v>352</v>
       </c>
       <c r="C4" t="s" s="45">
         <v>68</v>
       </c>
       <c r="D4" t="s" s="45">
-        <v>334</v>
+        <v>353</v>
       </c>
       <c r="E4" t="s" s="45">
         <v>66</v>
@@ -27847,13 +28016,13 @@
         <v>64</v>
       </c>
       <c r="B5" t="s" s="47">
-        <v>335</v>
+        <v>354</v>
       </c>
       <c r="C5" t="s" s="47">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="D5" t="s" s="47">
-        <v>337</v>
+        <v>356</v>
       </c>
       <c r="E5" t="s" s="47">
         <v>74</v>
@@ -27873,13 +28042,13 @@
         <v>64</v>
       </c>
       <c r="B6" t="s" s="45">
-        <v>338</v>
+        <v>357</v>
       </c>
       <c r="C6" t="s" s="45">
-        <v>339</v>
+        <v>358</v>
       </c>
       <c r="D6" t="s" s="45">
-        <v>340</v>
+        <v>359</v>
       </c>
       <c r="E6" t="s" s="45">
         <v>83</v>
@@ -27899,13 +28068,13 @@
         <v>64</v>
       </c>
       <c r="B7" t="s" s="47">
-        <v>341</v>
+        <v>360</v>
       </c>
       <c r="C7" t="s" s="47">
         <v>95</v>
       </c>
       <c r="D7" t="s" s="47">
-        <v>342</v>
+        <v>361</v>
       </c>
       <c r="E7" t="s" s="47">
         <v>92</v>
@@ -27925,13 +28094,13 @@
         <v>64</v>
       </c>
       <c r="B8" t="s" s="45">
-        <v>343</v>
+        <v>362</v>
       </c>
       <c r="C8" t="s" s="45">
         <v>106</v>
       </c>
       <c r="D8" t="s" s="45">
-        <v>344</v>
+        <v>363</v>
       </c>
       <c r="E8" t="s" s="45">
         <v>103</v>
@@ -27951,13 +28120,13 @@
         <v>64</v>
       </c>
       <c r="B9" t="s" s="47">
-        <v>345</v>
+        <v>364</v>
       </c>
       <c r="C9" t="s" s="47">
         <v>113</v>
       </c>
       <c r="D9" t="s" s="47">
-        <v>346</v>
+        <v>365</v>
       </c>
       <c r="E9" t="s" s="47">
         <v>111</v>
@@ -27977,13 +28146,13 @@
         <v>64</v>
       </c>
       <c r="B10" t="s" s="45">
-        <v>347</v>
+        <v>366</v>
       </c>
       <c r="C10" t="s" s="45">
-        <v>348</v>
+        <v>367</v>
       </c>
       <c r="D10" t="s" s="45">
-        <v>349</v>
+        <v>368</v>
       </c>
       <c r="E10" t="s" s="45">
         <v>73</v>
@@ -28003,13 +28172,13 @@
         <v>64</v>
       </c>
       <c r="B11" t="s" s="47">
-        <v>350</v>
+        <v>369</v>
       </c>
       <c r="C11" t="s" s="47">
         <v>132</v>
       </c>
       <c r="D11" t="s" s="47">
-        <v>351</v>
+        <v>370</v>
       </c>
       <c r="E11" t="s" s="47">
         <v>129</v>
@@ -28029,13 +28198,13 @@
         <v>64</v>
       </c>
       <c r="B12" t="s" s="45">
-        <v>352</v>
+        <v>371</v>
       </c>
       <c r="C12" t="s" s="45">
         <v>141</v>
       </c>
       <c r="D12" t="s" s="45">
-        <v>353</v>
+        <v>372</v>
       </c>
       <c r="E12" t="s" s="45">
         <v>65</v>
@@ -28092,7 +28261,7 @@
   <sheetData>
     <row r="1" ht="15.55" customHeight="1">
       <c r="A1" t="s" s="64">
-        <v>355</v>
+        <v>374</v>
       </c>
       <c r="B1" s="64"/>
       <c r="C1" s="64"/>
@@ -28107,19 +28276,19 @@
     </row>
     <row r="2" ht="20.05" customHeight="1">
       <c r="A2" t="s" s="41">
-        <v>357</v>
+        <v>376</v>
       </c>
       <c r="B2" t="s" s="41">
         <v>33</v>
       </c>
       <c r="C2" t="s" s="41">
-        <v>358</v>
+        <v>377</v>
       </c>
       <c r="D2" t="s" s="41">
         <v>15</v>
       </c>
       <c r="E2" t="s" s="41">
-        <v>359</v>
+        <v>378</v>
       </c>
       <c r="F2" t="s" s="41">
         <v>41</v>
@@ -28142,7 +28311,7 @@
     </row>
     <row r="3" ht="14.65" customHeight="1">
       <c r="A3" t="s" s="51">
-        <v>360</v>
+        <v>379</v>
       </c>
       <c r="B3" t="s" s="53">
         <v>50</v>
@@ -28151,31 +28320,31 @@
         <v>46281.958333333343</v>
       </c>
       <c r="D3" t="s" s="53">
-        <v>361</v>
+        <v>380</v>
       </c>
       <c r="E3" t="s" s="53">
-        <v>362</v>
+        <v>381</v>
       </c>
       <c r="F3" t="s" s="53">
         <v>58</v>
       </c>
       <c r="G3" t="s" s="53">
-        <v>363</v>
+        <v>382</v>
       </c>
       <c r="H3" t="s" s="53">
-        <v>363</v>
+        <v>382</v>
       </c>
       <c r="I3" s="54"/>
       <c r="J3" t="s" s="53">
-        <v>364</v>
+        <v>383</v>
       </c>
       <c r="K3" t="s" s="53">
-        <v>365</v>
+        <v>384</v>
       </c>
     </row>
     <row r="4" ht="11.55" customHeight="1">
       <c r="A4" t="s" s="55">
-        <v>366</v>
+        <v>385</v>
       </c>
       <c r="B4" t="s" s="57">
         <v>66</v>
@@ -28184,10 +28353,10 @@
         <v>46282.458333333336</v>
       </c>
       <c r="D4" t="s" s="57">
-        <v>361</v>
+        <v>380</v>
       </c>
       <c r="E4" t="s" s="57">
-        <v>362</v>
+        <v>381</v>
       </c>
       <c r="F4" t="s" s="57">
         <v>58</v>
@@ -28196,15 +28365,15 @@
       <c r="H4" s="58"/>
       <c r="I4" s="58"/>
       <c r="J4" t="s" s="57">
-        <v>367</v>
+        <v>386</v>
       </c>
       <c r="K4" t="s" s="57">
-        <v>368</v>
+        <v>387</v>
       </c>
     </row>
     <row r="5" ht="11.55" customHeight="1">
       <c r="A5" t="s" s="55">
-        <v>369</v>
+        <v>388</v>
       </c>
       <c r="B5" t="s" s="60">
         <v>74</v>
@@ -28213,10 +28382,10 @@
         <v>46282.958333333336</v>
       </c>
       <c r="D5" t="s" s="60">
-        <v>361</v>
+        <v>380</v>
       </c>
       <c r="E5" t="s" s="60">
-        <v>362</v>
+        <v>381</v>
       </c>
       <c r="F5" t="s" s="60">
         <v>58</v>
@@ -28225,15 +28394,15 @@
       <c r="H5" s="61"/>
       <c r="I5" s="61"/>
       <c r="J5" t="s" s="60">
-        <v>370</v>
+        <v>389</v>
       </c>
       <c r="K5" t="s" s="60">
-        <v>371</v>
+        <v>390</v>
       </c>
     </row>
     <row r="6" ht="11.55" customHeight="1">
       <c r="A6" t="s" s="55">
-        <v>372</v>
+        <v>391</v>
       </c>
       <c r="B6" t="s" s="57">
         <v>83</v>
@@ -28242,10 +28411,10 @@
         <v>46282.958333333336</v>
       </c>
       <c r="D6" t="s" s="57">
-        <v>361</v>
+        <v>380</v>
       </c>
       <c r="E6" t="s" s="57">
-        <v>362</v>
+        <v>381</v>
       </c>
       <c r="F6" t="s" s="57">
         <v>58</v>
@@ -28254,15 +28423,15 @@
       <c r="H6" s="58"/>
       <c r="I6" s="58"/>
       <c r="J6" t="s" s="57">
-        <v>373</v>
+        <v>392</v>
       </c>
       <c r="K6" t="s" s="57">
-        <v>374</v>
+        <v>393</v>
       </c>
     </row>
     <row r="7" ht="11.55" customHeight="1">
       <c r="A7" t="s" s="55">
-        <v>375</v>
+        <v>394</v>
       </c>
       <c r="B7" t="s" s="60">
         <v>92</v>
@@ -28271,10 +28440,10 @@
         <v>46283</v>
       </c>
       <c r="D7" t="s" s="60">
-        <v>361</v>
+        <v>380</v>
       </c>
       <c r="E7" t="s" s="60">
-        <v>362</v>
+        <v>381</v>
       </c>
       <c r="F7" t="s" s="60">
         <v>58</v>
@@ -28283,48 +28452,54 @@
       <c r="H7" s="61"/>
       <c r="I7" s="61"/>
       <c r="J7" t="s" s="60">
-        <v>376</v>
+        <v>395</v>
       </c>
       <c r="K7" t="s" s="60">
-        <v>377</v>
+        <v>396</v>
       </c>
     </row>
     <row r="8" ht="11.55" customHeight="1">
       <c r="A8" t="s" s="55">
-        <v>378</v>
+        <v>397</v>
       </c>
       <c r="B8" t="s" s="57">
         <v>103</v>
       </c>
-      <c r="C8" s="66"/>
+      <c r="C8" s="66">
+        <v>46283</v>
+      </c>
       <c r="D8" t="s" s="57">
-        <v>361</v>
+        <v>380</v>
       </c>
       <c r="E8" t="s" s="57">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="F8" t="s" s="57">
-        <v>98</v>
+        <v>58</v>
       </c>
       <c r="G8" s="58"/>
       <c r="H8" s="58"/>
       <c r="I8" s="58"/>
-      <c r="J8" s="58"/>
-      <c r="K8" s="58"/>
+      <c r="J8" t="s" s="57">
+        <v>398</v>
+      </c>
+      <c r="K8" t="s" s="57">
+        <v>399</v>
+      </c>
     </row>
     <row r="9" ht="11.55" customHeight="1">
       <c r="A9" t="s" s="55">
-        <v>380</v>
+        <v>400</v>
       </c>
       <c r="B9" t="s" s="60">
         <v>111</v>
       </c>
       <c r="C9" s="67"/>
       <c r="D9" t="s" s="60">
-        <v>361</v>
+        <v>380</v>
       </c>
       <c r="E9" t="s" s="60">
-        <v>379</v>
+        <v>401</v>
       </c>
       <c r="F9" t="s" s="60">
         <v>98</v>
@@ -28337,17 +28512,17 @@
     </row>
     <row r="10" ht="11.55" customHeight="1">
       <c r="A10" t="s" s="55">
-        <v>381</v>
+        <v>402</v>
       </c>
       <c r="B10" t="s" s="57">
         <v>73</v>
       </c>
       <c r="C10" s="66"/>
       <c r="D10" t="s" s="57">
-        <v>361</v>
+        <v>380</v>
       </c>
       <c r="E10" t="s" s="57">
-        <v>379</v>
+        <v>401</v>
       </c>
       <c r="F10" t="s" s="57">
         <v>98</v>
@@ -28360,17 +28535,17 @@
     </row>
     <row r="11" ht="11.55" customHeight="1">
       <c r="A11" t="s" s="55">
-        <v>382</v>
+        <v>403</v>
       </c>
       <c r="B11" t="s" s="60">
         <v>129</v>
       </c>
       <c r="C11" s="67"/>
       <c r="D11" t="s" s="60">
-        <v>361</v>
+        <v>380</v>
       </c>
       <c r="E11" t="s" s="60">
-        <v>379</v>
+        <v>401</v>
       </c>
       <c r="F11" t="s" s="60">
         <v>98</v>
@@ -28383,7 +28558,7 @@
     </row>
     <row r="12" ht="11.55" customHeight="1">
       <c r="A12" t="s" s="55">
-        <v>383</v>
+        <v>404</v>
       </c>
       <c r="B12" t="s" s="57">
         <v>65</v>
@@ -28392,10 +28567,10 @@
         <v>46282.958333333336</v>
       </c>
       <c r="D12" t="s" s="57">
-        <v>361</v>
+        <v>380</v>
       </c>
       <c r="E12" t="s" s="57">
-        <v>362</v>
+        <v>381</v>
       </c>
       <c r="F12" t="s" s="57">
         <v>98</v>
@@ -28404,15 +28579,15 @@
       <c r="H12" s="58"/>
       <c r="I12" s="58"/>
       <c r="J12" t="s" s="57">
-        <v>384</v>
+        <v>405</v>
       </c>
       <c r="K12" t="s" s="57">
-        <v>385</v>
+        <v>406</v>
       </c>
     </row>
     <row r="13" ht="11.55" customHeight="1">
       <c r="A13" t="s" s="55">
-        <v>386</v>
+        <v>407</v>
       </c>
       <c r="B13" t="s" s="60">
         <v>50</v>
@@ -28421,29 +28596,29 @@
         <v>46282.958333333336</v>
       </c>
       <c r="D13" t="s" s="60">
-        <v>361</v>
+        <v>380</v>
       </c>
       <c r="E13" t="s" s="60">
-        <v>362</v>
+        <v>381</v>
       </c>
       <c r="F13" t="s" s="60">
         <v>58</v>
       </c>
       <c r="G13" t="s" s="60">
-        <v>363</v>
+        <v>382</v>
       </c>
       <c r="H13" t="s" s="60">
-        <v>363</v>
+        <v>382</v>
       </c>
       <c r="I13" s="61"/>
       <c r="J13" s="60"/>
       <c r="K13" t="s" s="60">
-        <v>387</v>
+        <v>408</v>
       </c>
     </row>
     <row r="14" ht="11.55" customHeight="1">
       <c r="A14" t="s" s="55">
-        <v>388</v>
+        <v>409</v>
       </c>
       <c r="B14" t="s" s="57">
         <v>147</v>
@@ -28452,10 +28627,10 @@
         <v>46283.958333333336</v>
       </c>
       <c r="D14" t="s" s="57">
-        <v>361</v>
+        <v>380</v>
       </c>
       <c r="E14" t="s" s="57">
-        <v>362</v>
+        <v>381</v>
       </c>
       <c r="F14" t="s" s="57">
         <v>58</v>
@@ -28464,10 +28639,10 @@
       <c r="H14" s="58"/>
       <c r="I14" s="58"/>
       <c r="J14" t="s" s="57">
-        <v>389</v>
+        <v>410</v>
       </c>
       <c r="K14" t="s" s="57">
-        <v>390</v>
+        <v>411</v>
       </c>
     </row>
     <row r="15" ht="11.55" customHeight="1">
@@ -41340,7 +41515,7 @@
   <sheetData>
     <row r="1" ht="15.55" customHeight="1">
       <c r="A1" t="s" s="36">
-        <v>392</v>
+        <v>413</v>
       </c>
       <c r="B1" s="37"/>
       <c r="C1" s="38"/>
@@ -41370,10 +41545,10 @@
         <v>33</v>
       </c>
       <c r="D2" t="s" s="41">
-        <v>357</v>
+        <v>376</v>
       </c>
       <c r="E2" t="s" s="41">
-        <v>393</v>
+        <v>414</v>
       </c>
       <c r="F2" t="s" s="41">
         <v>38</v>
@@ -41388,7 +41563,7 @@
         <v>15</v>
       </c>
       <c r="J2" t="s" s="41">
-        <v>394</v>
+        <v>415</v>
       </c>
       <c r="K2" t="s" s="41">
         <v>159</v>
@@ -41400,10 +41575,10 @@
         <v>160</v>
       </c>
       <c r="N2" t="s" s="41">
-        <v>395</v>
+        <v>416</v>
       </c>
       <c r="O2" t="s" s="41">
-        <v>396</v>
+        <v>417</v>
       </c>
       <c r="P2" t="s" s="41">
         <v>163</v>
@@ -60413,7 +60588,7 @@
   <sheetData>
     <row r="1" ht="15.55" customHeight="1">
       <c r="A1" t="s" s="36">
-        <v>397</v>
+        <v>418</v>
       </c>
       <c r="B1" s="37"/>
       <c r="C1" s="38"/>
@@ -60428,13 +60603,13 @@
         <v>33</v>
       </c>
       <c r="B2" t="s" s="41">
-        <v>398</v>
+        <v>419</v>
       </c>
       <c r="C2" t="s" s="41">
-        <v>399</v>
+        <v>420</v>
       </c>
       <c r="D2" t="s" s="41">
-        <v>400</v>
+        <v>421</v>
       </c>
       <c r="E2" t="s" s="41">
         <v>42</v>
@@ -60455,19 +60630,19 @@
         <v>57</v>
       </c>
       <c r="C3" t="s" s="43">
-        <v>401</v>
+        <v>422</v>
       </c>
       <c r="D3" t="s" s="43">
-        <v>402</v>
+        <v>423</v>
       </c>
       <c r="E3" t="s" s="43">
-        <v>403</v>
+        <v>424</v>
       </c>
       <c r="F3" t="s" s="43">
-        <v>404</v>
+        <v>425</v>
       </c>
       <c r="G3" t="s" s="43">
-        <v>405</v>
+        <v>426</v>
       </c>
       <c r="H3" s="44"/>
     </row>
@@ -60479,19 +60654,19 @@
         <v>57</v>
       </c>
       <c r="C4" t="s" s="45">
-        <v>401</v>
+        <v>422</v>
       </c>
       <c r="D4" t="s" s="45">
-        <v>406</v>
+        <v>427</v>
       </c>
       <c r="E4" t="s" s="45">
-        <v>403</v>
+        <v>424</v>
       </c>
       <c r="F4" t="s" s="45">
-        <v>404</v>
+        <v>425</v>
       </c>
       <c r="G4" t="s" s="45">
-        <v>407</v>
+        <v>428</v>
       </c>
       <c r="H4" s="46"/>
     </row>
@@ -60503,19 +60678,19 @@
         <v>57</v>
       </c>
       <c r="C5" t="s" s="47">
-        <v>401</v>
+        <v>422</v>
       </c>
       <c r="D5" t="s" s="47">
-        <v>408</v>
+        <v>429</v>
       </c>
       <c r="E5" t="s" s="47">
-        <v>403</v>
+        <v>424</v>
       </c>
       <c r="F5" t="s" s="47">
-        <v>404</v>
+        <v>425</v>
       </c>
       <c r="G5" t="s" s="47">
-        <v>409</v>
+        <v>430</v>
       </c>
       <c r="H5" s="48"/>
     </row>
@@ -60527,19 +60702,19 @@
         <v>57</v>
       </c>
       <c r="C6" t="s" s="45">
-        <v>401</v>
+        <v>422</v>
       </c>
       <c r="D6" t="s" s="45">
-        <v>408</v>
+        <v>429</v>
       </c>
       <c r="E6" t="s" s="45">
-        <v>403</v>
+        <v>424</v>
       </c>
       <c r="F6" t="s" s="45">
-        <v>404</v>
+        <v>425</v>
       </c>
       <c r="G6" t="s" s="45">
-        <v>410</v>
+        <v>431</v>
       </c>
       <c r="H6" s="46"/>
     </row>
@@ -60551,19 +60726,19 @@
         <v>57</v>
       </c>
       <c r="C7" t="s" s="47">
-        <v>401</v>
+        <v>422</v>
       </c>
       <c r="D7" t="s" s="47">
-        <v>411</v>
+        <v>432</v>
       </c>
       <c r="E7" t="s" s="47">
-        <v>403</v>
+        <v>424</v>
       </c>
       <c r="F7" t="s" s="47">
-        <v>404</v>
+        <v>425</v>
       </c>
       <c r="G7" t="s" s="47">
-        <v>412</v>
+        <v>433</v>
       </c>
       <c r="H7" s="48"/>
     </row>
@@ -60575,19 +60750,19 @@
         <v>57</v>
       </c>
       <c r="C8" t="s" s="45">
-        <v>401</v>
+        <v>422</v>
       </c>
       <c r="D8" t="s" s="45">
-        <v>413</v>
+        <v>434</v>
       </c>
       <c r="E8" t="s" s="45">
-        <v>403</v>
+        <v>424</v>
       </c>
       <c r="F8" t="s" s="45">
-        <v>404</v>
+        <v>425</v>
       </c>
       <c r="G8" t="s" s="45">
-        <v>414</v>
+        <v>435</v>
       </c>
       <c r="H8" s="46"/>
     </row>
@@ -60599,19 +60774,19 @@
         <v>57</v>
       </c>
       <c r="C9" t="s" s="47">
-        <v>401</v>
+        <v>422</v>
       </c>
       <c r="D9" t="s" s="47">
-        <v>413</v>
+        <v>434</v>
       </c>
       <c r="E9" t="s" s="47">
-        <v>403</v>
+        <v>424</v>
       </c>
       <c r="F9" t="s" s="47">
-        <v>404</v>
+        <v>425</v>
       </c>
       <c r="G9" t="s" s="47">
-        <v>415</v>
+        <v>436</v>
       </c>
       <c r="H9" s="48"/>
     </row>
@@ -60623,19 +60798,19 @@
         <v>57</v>
       </c>
       <c r="C10" t="s" s="45">
-        <v>401</v>
+        <v>422</v>
       </c>
       <c r="D10" t="s" s="45">
-        <v>416</v>
+        <v>437</v>
       </c>
       <c r="E10" t="s" s="45">
-        <v>403</v>
+        <v>424</v>
       </c>
       <c r="F10" t="s" s="45">
-        <v>404</v>
+        <v>425</v>
       </c>
       <c r="G10" t="s" s="45">
-        <v>417</v>
+        <v>438</v>
       </c>
       <c r="H10" s="46"/>
     </row>
@@ -60647,19 +60822,19 @@
         <v>134</v>
       </c>
       <c r="C11" t="s" s="47">
-        <v>401</v>
+        <v>422</v>
       </c>
       <c r="D11" t="s" s="47">
-        <v>418</v>
+        <v>439</v>
       </c>
       <c r="E11" t="s" s="47">
-        <v>403</v>
+        <v>424</v>
       </c>
       <c r="F11" t="s" s="47">
-        <v>404</v>
+        <v>425</v>
       </c>
       <c r="G11" t="s" s="47">
-        <v>419</v>
+        <v>440</v>
       </c>
       <c r="H11" s="48"/>
     </row>
@@ -60671,19 +60846,19 @@
         <v>57</v>
       </c>
       <c r="C12" t="s" s="45">
-        <v>401</v>
+        <v>422</v>
       </c>
       <c r="D12" t="s" s="45">
-        <v>408</v>
+        <v>429</v>
       </c>
       <c r="E12" t="s" s="45">
-        <v>403</v>
+        <v>424</v>
       </c>
       <c r="F12" t="s" s="45">
-        <v>404</v>
+        <v>425</v>
       </c>
       <c r="G12" t="s" s="45">
-        <v>420</v>
+        <v>441</v>
       </c>
       <c r="H12" s="46"/>
     </row>
@@ -70609,7 +70784,7 @@
   <sheetData>
     <row r="1" ht="19.45" customHeight="1">
       <c r="A1" t="s" s="72">
-        <v>422</v>
+        <v>443</v>
       </c>
       <c r="B1" s="73"/>
       <c r="C1" s="73"/>
@@ -70647,7 +70822,7 @@
     </row>
     <row r="3" ht="19.55" customHeight="1">
       <c r="A3" t="s" s="76">
-        <v>423</v>
+        <v>444</v>
       </c>
       <c r="B3" s="77">
         <f>COUNTA('Test Cases'!A3:A1000)</f>
@@ -70670,11 +70845,11 @@
     </row>
     <row r="4" ht="19.55" customHeight="1">
       <c r="A4" t="s" s="76">
-        <v>424</v>
+        <v>445</v>
       </c>
       <c r="B4" s="77">
         <f>COUNTIF('Test Execution - Test Execution'!F3:F1001,"Pass")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C4" s="22"/>
       <c r="D4" s="20"/>
@@ -70693,7 +70868,7 @@
     </row>
     <row r="5" ht="19.55" customHeight="1">
       <c r="A5" t="s" s="76">
-        <v>425</v>
+        <v>446</v>
       </c>
       <c r="B5" s="77">
         <f>COUNTIF('Test Execution - Test Execution'!F3:F1001,"Fail")</f>
@@ -70716,7 +70891,7 @@
     </row>
     <row r="6" ht="19.55" customHeight="1">
       <c r="A6" t="s" s="76">
-        <v>426</v>
+        <v>447</v>
       </c>
       <c r="B6" s="77">
         <f>COUNTIF('Test Execution - Test Execution'!F3:F1001,"Blocked")</f>
@@ -70739,7 +70914,7 @@
     </row>
     <row r="7" ht="19.55" customHeight="1">
       <c r="A7" t="s" s="76">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="B7" s="77">
         <f>COUNTIF('Test Execution - Test Execution'!F3:F1001,"Skipped")</f>
@@ -70766,7 +70941,7 @@
       </c>
       <c r="B8" s="77">
         <f>COUNTIF('Test Execution - Test Execution'!F3:F1001,"Not Run")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C8" s="22"/>
       <c r="D8" s="20"/>
@@ -70785,7 +70960,7 @@
     </row>
     <row r="9" ht="19.55" customHeight="1">
       <c r="A9" t="s" s="76">
-        <v>403</v>
+        <v>424</v>
       </c>
       <c r="B9" s="77">
         <f>COUNTIF('Automation Mapping'!E3:E1000,"Automated")</f>
@@ -70808,7 +70983,7 @@
     </row>
     <row r="10" ht="19.55" customHeight="1">
       <c r="A10" t="s" s="76">
-        <v>428</v>
+        <v>449</v>
       </c>
       <c r="B10" s="77">
         <f>COUNTIF('Defects'!H3:H1000,"Open")</f>
@@ -70831,7 +71006,7 @@
     </row>
     <row r="11" ht="19.55" customHeight="1">
       <c r="A11" t="s" s="76">
-        <v>429</v>
+        <v>450</v>
       </c>
       <c r="B11" s="77">
         <f>COUNTIF('Defects'!F3:F1000,"Critical")</f>
@@ -70854,7 +71029,7 @@
     </row>
     <row r="12" ht="19.55" customHeight="1">
       <c r="A12" t="s" s="76">
-        <v>430</v>
+        <v>451</v>
       </c>
       <c r="B12" s="78">
         <f>IF(B3=0,0,B3/B3)</f>
@@ -70877,11 +71052,11 @@
     </row>
     <row r="13" ht="19.55" customHeight="1">
       <c r="A13" t="s" s="76">
-        <v>431</v>
+        <v>452</v>
       </c>
       <c r="B13" s="78">
         <f>IF(COUNTA('Automation Mapping'!A3:A1000)=0,0,B8/COUNTA('Automation Mapping'!A3:A1000))</f>
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="C13" s="22"/>
       <c r="D13" s="20"/>
@@ -70979,7 +71154,7 @@
       </c>
       <c r="E18" s="80">
         <f>COUNTIF('Test Execution - Test Execution'!F3:F1001,"Pass")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F18" s="20"/>
       <c r="G18" s="20"/>
@@ -70993,7 +71168,7 @@
       <c r="J18" s="20"/>
       <c r="K18" s="20"/>
       <c r="L18" t="s" s="79">
-        <v>432</v>
+        <v>453</v>
       </c>
       <c r="M18" s="81">
         <f>COUNTIF('Defects'!F3:F1000,"Critical")</f>
@@ -71008,7 +71183,7 @@
       <c r="B19" s="20"/>
       <c r="C19" s="20"/>
       <c r="D19" t="s" s="79">
-        <v>433</v>
+        <v>454</v>
       </c>
       <c r="E19" s="80">
         <f>COUNTIF('Test Execution - Test Execution'!F3:F1001,"Fail")</f>
@@ -71041,7 +71216,7 @@
       <c r="B20" s="20"/>
       <c r="C20" s="20"/>
       <c r="D20" t="s" s="79">
-        <v>426</v>
+        <v>447</v>
       </c>
       <c r="E20" s="80">
         <f>COUNTIF('Test Execution - Test Execution'!F3:F1001,"Blocked")</f>
@@ -71074,7 +71249,7 @@
       <c r="B21" s="20"/>
       <c r="C21" s="20"/>
       <c r="D21" t="s" s="79">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="E21" s="80">
         <f>COUNTIF('Test Execution - Test Execution'!F3:F1001,"Skipped")</f>
@@ -71092,7 +71267,7 @@
       <c r="J21" s="20"/>
       <c r="K21" s="20"/>
       <c r="L21" t="s" s="79">
-        <v>434</v>
+        <v>455</v>
       </c>
       <c r="M21" s="81">
         <f>COUNTIF('Defects'!F3:F1000,"Low")</f>
@@ -71111,7 +71286,7 @@
       </c>
       <c r="E22" s="85">
         <f>COUNTIF('Test Execution - Test Execution'!F3:F1001,"Not Run")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F22" s="83"/>
       <c r="G22" s="83"/>

</xml_diff>